<commit_message>
Improve cockpit: exclude outliers from comparison, show date basis, surface permit/keishin data
- 比較対象外フラグ（Excel列・永続化）でHIRAYAMA等をランキング/チャート/業界内比較から除外（DBには残し一覧では「比較対象外」バッジ表示）
- 被保険者数・売上・自己資本の増減に基準日を明示（雇用は日付付きスナップショットを優先、チャートのツールチップにも基準を表示）
- 許可業種・有効期間・経審P点・自動取得日を企業カードに表示。経審/許可リンクを「公式確認」に整理
- 自社サマリーの業界内ポジションも比較対象外を除外して算出

https://claude.ai/code/session_01KdqRhSedTB9yYtspSnu4Ax
</commit_message>
<xml_diff>
--- a/cockpit-7r2x9k/data/companies.xlsx
+++ b/cockpit-7r2x9k/data/companies.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P78"/>
+  <dimension ref="A1:Q78"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -448,6 +448,9 @@
       <c r="P1" t="str">
         <v>自社</v>
       </c>
+      <c r="Q1" t="str">
+        <v>比較対象外</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -498,6 +501,9 @@
       <c r="P2" t="str">
         <v/>
       </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -548,6 +554,9 @@
       <c r="P3" t="str">
         <v/>
       </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -598,6 +607,9 @@
       <c r="P4" t="str">
         <v/>
       </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -648,6 +660,9 @@
       <c r="P5" t="str">
         <v/>
       </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -698,6 +713,9 @@
       <c r="P6" t="str">
         <v>○</v>
       </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -748,6 +766,9 @@
       <c r="P7" t="str">
         <v/>
       </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -798,6 +819,9 @@
       <c r="P8" t="str">
         <v/>
       </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -848,6 +872,9 @@
       <c r="P9" t="str">
         <v/>
       </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -898,6 +925,9 @@
       <c r="P10" t="str">
         <v/>
       </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -948,6 +978,9 @@
       <c r="P11" t="str">
         <v/>
       </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -998,6 +1031,9 @@
       <c r="P12" t="str">
         <v/>
       </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1048,6 +1084,9 @@
       <c r="P13" t="str">
         <v/>
       </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1098,6 +1137,9 @@
       <c r="P14" t="str">
         <v/>
       </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1148,6 +1190,9 @@
       <c r="P15" t="str">
         <v/>
       </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1198,6 +1243,9 @@
       <c r="P16" t="str">
         <v/>
       </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1248,6 +1296,9 @@
       <c r="P17" t="str">
         <v/>
       </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1298,6 +1349,9 @@
       <c r="P18" t="str">
         <v/>
       </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1348,6 +1402,9 @@
       <c r="P19" t="str">
         <v/>
       </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1398,6 +1455,9 @@
       <c r="P20" t="str">
         <v/>
       </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1448,6 +1508,9 @@
       <c r="P21" t="str">
         <v/>
       </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1498,6 +1561,9 @@
       <c r="P22" t="str">
         <v/>
       </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1548,6 +1614,9 @@
       <c r="P23" t="str">
         <v/>
       </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1598,6 +1667,9 @@
       <c r="P24" t="str">
         <v/>
       </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1648,6 +1720,9 @@
       <c r="P25" t="str">
         <v/>
       </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1698,6 +1773,9 @@
       <c r="P26" t="str">
         <v/>
       </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1748,6 +1826,9 @@
       <c r="P27" t="str">
         <v/>
       </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1798,6 +1879,9 @@
       <c r="P28" t="str">
         <v/>
       </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1848,6 +1932,9 @@
       <c r="P29" t="str">
         <v/>
       </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1898,6 +1985,9 @@
       <c r="P30" t="str">
         <v/>
       </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1948,6 +2038,9 @@
       <c r="P31" t="str">
         <v/>
       </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1998,6 +2091,9 @@
       <c r="P32" t="str">
         <v/>
       </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -2048,6 +2144,9 @@
       <c r="P33" t="str">
         <v/>
       </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2098,6 +2197,9 @@
       <c r="P34" t="str">
         <v/>
       </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2148,6 +2250,9 @@
       <c r="P35" t="str">
         <v/>
       </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -2198,6 +2303,9 @@
       <c r="P36" t="str">
         <v/>
       </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2248,6 +2356,9 @@
       <c r="P37" t="str">
         <v/>
       </c>
+      <c r="Q37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -2298,6 +2409,9 @@
       <c r="P38" t="str">
         <v/>
       </c>
+      <c r="Q38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -2348,6 +2462,9 @@
       <c r="P39" t="str">
         <v/>
       </c>
+      <c r="Q39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -2398,6 +2515,9 @@
       <c r="P40" t="str">
         <v/>
       </c>
+      <c r="Q40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2448,6 +2568,9 @@
       <c r="P41" t="str">
         <v/>
       </c>
+      <c r="Q41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -2498,6 +2621,9 @@
       <c r="P42" t="str">
         <v/>
       </c>
+      <c r="Q42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2548,6 +2674,9 @@
       <c r="P43" t="str">
         <v/>
       </c>
+      <c r="Q43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -2598,6 +2727,9 @@
       <c r="P44" t="str">
         <v/>
       </c>
+      <c r="Q44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2648,6 +2780,9 @@
       <c r="P45" t="str">
         <v/>
       </c>
+      <c r="Q45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2698,6 +2833,9 @@
       <c r="P46" t="str">
         <v/>
       </c>
+      <c r="Q46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2748,6 +2886,9 @@
       <c r="P47" t="str">
         <v/>
       </c>
+      <c r="Q47" t="str">
+        <v>○</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2798,6 +2939,9 @@
       <c r="P48" t="str">
         <v/>
       </c>
+      <c r="Q48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2848,6 +2992,9 @@
       <c r="P49" t="str">
         <v/>
       </c>
+      <c r="Q49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2898,6 +3045,9 @@
       <c r="P50" t="str">
         <v/>
       </c>
+      <c r="Q50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2948,6 +3098,9 @@
       <c r="P51" t="str">
         <v/>
       </c>
+      <c r="Q51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2998,6 +3151,9 @@
       <c r="P52" t="str">
         <v/>
       </c>
+      <c r="Q52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -3048,6 +3204,9 @@
       <c r="P53" t="str">
         <v/>
       </c>
+      <c r="Q53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -3098,6 +3257,9 @@
       <c r="P54" t="str">
         <v/>
       </c>
+      <c r="Q54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -3148,6 +3310,9 @@
       <c r="P55" t="str">
         <v/>
       </c>
+      <c r="Q55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -3198,6 +3363,9 @@
       <c r="P56" t="str">
         <v/>
       </c>
+      <c r="Q56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -3248,6 +3416,9 @@
       <c r="P57" t="str">
         <v/>
       </c>
+      <c r="Q57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -3298,6 +3469,9 @@
       <c r="P58" t="str">
         <v/>
       </c>
+      <c r="Q58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -3348,6 +3522,9 @@
       <c r="P59" t="str">
         <v/>
       </c>
+      <c r="Q59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -3398,6 +3575,9 @@
       <c r="P60" t="str">
         <v/>
       </c>
+      <c r="Q60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -3448,6 +3628,9 @@
       <c r="P61" t="str">
         <v/>
       </c>
+      <c r="Q61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -3498,6 +3681,9 @@
       <c r="P62" t="str">
         <v/>
       </c>
+      <c r="Q62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -3548,6 +3734,9 @@
       <c r="P63" t="str">
         <v/>
       </c>
+      <c r="Q63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -3598,6 +3787,9 @@
       <c r="P64" t="str">
         <v/>
       </c>
+      <c r="Q64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -3648,6 +3840,9 @@
       <c r="P65" t="str">
         <v/>
       </c>
+      <c r="Q65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -3698,6 +3893,9 @@
       <c r="P66" t="str">
         <v/>
       </c>
+      <c r="Q66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -3748,6 +3946,9 @@
       <c r="P67" t="str">
         <v/>
       </c>
+      <c r="Q67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -3798,6 +3999,9 @@
       <c r="P68" t="str">
         <v/>
       </c>
+      <c r="Q68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -3848,6 +4052,9 @@
       <c r="P69" t="str">
         <v/>
       </c>
+      <c r="Q69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -3898,6 +4105,9 @@
       <c r="P70" t="str">
         <v/>
       </c>
+      <c r="Q70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -3948,6 +4158,9 @@
       <c r="P71" t="str">
         <v/>
       </c>
+      <c r="Q71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -3998,6 +4211,9 @@
       <c r="P72" t="str">
         <v/>
       </c>
+      <c r="Q72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -4048,6 +4264,9 @@
       <c r="P73" t="str">
         <v/>
       </c>
+      <c r="Q73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -4098,6 +4317,9 @@
       <c r="P74" t="str">
         <v/>
       </c>
+      <c r="Q74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -4148,6 +4370,9 @@
       <c r="P75" t="str">
         <v/>
       </c>
+      <c r="Q75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -4198,6 +4423,9 @@
       <c r="P76" t="str">
         <v/>
       </c>
+      <c r="Q76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -4248,6 +4476,9 @@
       <c r="P77" t="str">
         <v/>
       </c>
+      <c r="Q77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -4298,10 +4529,13 @@
       <c r="P78" t="str">
         <v/>
       </c>
+      <c r="Q78" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q78"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>